<commit_message>
Update batch_27.xlsx with new content and improvements
</commit_message>
<xml_diff>
--- a/batch_notes/27/batch_27.xlsx
+++ b/batch_notes/27/batch_27.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/shira_2/__work__/acciojob/modules/sql/postgresql/batch_notes/27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F41B00F-7B4E-2748-B3A3-446F4AD8F196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41BCC7D-7273-254A-A7A1-38CC97F55CA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="-2480" windowWidth="38400" windowHeight="21600" activeTab="15" xr2:uid="{43D057EC-24A4-D14F-BD50-FDFE67984E9E}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1278" uniqueCount="666">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1280" uniqueCount="667">
   <si>
     <t>RDBMS</t>
   </si>
@@ -2077,6 +2077,9 @@
   </si>
   <si>
     <t>cat4</t>
+  </si>
+  <si>
+    <t>cust_id 50 =&gt; 5,6,8</t>
   </si>
 </sst>
 </file>
@@ -2400,7 +2403,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -2474,6 +2477,13 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2492,15 +2502,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -7691,6 +7693,332 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>686713</xdr:colOff>
+      <xdr:row>116</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1038441</xdr:colOff>
+      <xdr:row>168</xdr:row>
+      <xdr:rowOff>19700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1" descr="How to Read Postgres EXPLAIN: A Guide to Scan... | Crunchy Data Blog">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE5F34FB-9D3D-3808-80D2-C493CF435ED2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="686713" y="23787100"/>
+          <a:ext cx="7120828" cy="10548000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>68920</xdr:colOff>
+      <xdr:row>179</xdr:row>
+      <xdr:rowOff>118080</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>84040</xdr:colOff>
+      <xdr:row>179</xdr:row>
+      <xdr:rowOff>147240</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="3" name="Ink 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DD9533F-45D9-A559-51DE-65143F4362F7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="1923120" y="36694080"/>
+            <a:ext cx="15120" cy="29160"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="3" name="Ink 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DD9533F-45D9-A559-51DE-65143F4362F7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="1918800" y="36689760"/>
+              <a:ext cx="23760" cy="37800"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>160360</xdr:colOff>
+      <xdr:row>181</xdr:row>
+      <xdr:rowOff>116840</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>222700</xdr:colOff>
+      <xdr:row>185</xdr:row>
+      <xdr:rowOff>184960</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="12" name="Ink 11">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C4CC508-AA12-FD0C-19C4-6CCE0BA56A26}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="2014560" y="37124640"/>
+            <a:ext cx="2843640" cy="880920"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="12" name="Ink 11">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C4CC508-AA12-FD0C-19C4-6CCE0BA56A26}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2010240" y="37120320"/>
+              <a:ext cx="2852280" cy="889560"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>998620</xdr:colOff>
+      <xdr:row>172</xdr:row>
+      <xdr:rowOff>68180</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>493900</xdr:colOff>
+      <xdr:row>175</xdr:row>
+      <xdr:rowOff>25480</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="15" name="Ink 14">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{395C6C07-81FC-D7EF-A434-A8F14892AF18}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="1824120" y="35209080"/>
+            <a:ext cx="9553680" cy="579600"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="15" name="Ink 14">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{395C6C07-81FC-D7EF-A434-A8F14892AF18}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="1819800" y="35204760"/>
+              <a:ext cx="9562320" cy="588240"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>427480</xdr:colOff>
+      <xdr:row>175</xdr:row>
+      <xdr:rowOff>71920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>431300</xdr:colOff>
+      <xdr:row>177</xdr:row>
+      <xdr:rowOff>11840</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="18" name="Ink 17">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C34F1CE-92B3-FA88-6E6E-BB4B918E2DF6}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="2281680" y="35835120"/>
+            <a:ext cx="8068320" cy="346320"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="18" name="Ink 17">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C34F1CE-92B3-FA88-6E6E-BB4B918E2DF6}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="2277360" y="35830796"/>
+              <a:ext cx="8076960" cy="354969"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/ink/ink1.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
@@ -8470,6 +8798,121 @@
 </inkml:ink>
 </file>
 
+<file path=xl/ink/ink33.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-07-26T07:42:58.534"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 1 24575,'19'36'0,"-15"-24"0,15 20 0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink34.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-07-26T07:42:59.934"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">165 190 24575,'34'-17'0,"53"-7"0,-16 12 0,4 1 0,-17 0 0,4 1 0,17 1 0,10 0 0,-7 2 0,-7 2 0,-2-1 0,-8 1 0,4-2 0,-3 1 0,17-3 0,-9 1 0,3-5 0,-13 2 0,-25 5 0,11 6 0,14-4 0,1 4 0,-26 0 0,-7 0 0,-11 0 0,7 0 0,-1 0 0,2 3 0,-8-1 0,13 8 0,8 0 0,1 1 0,9-3 0,-21-2 0,0-3 0,9 5 0,-4-4 0,5 3 0,-15-5 0,-19-2 0,0-2 0,-4 3 0,-1-2 0,-2 3 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1533">2557 355 24575,'-16'-4'0,"-21"-2"0,-57 1 0,23 4 0,-5 2 0,3 2 0,-5 0 0,-5 0 0,-7 1 0,7 0 0,7-1 0,0 0 0,-4-1 0,-5 0 0,10-1 0,17-3 0,4 0 0,-20 1 0,5 1 0,0-5 0,7 4 0,-6 2 0,-9 4 0,3 0 0,20-4 0,0 0 0,-37 6 0,13-1 0,46-5 0,-38 3 0,25-4 0,-38 0 0,13 0 0,10-1 0,3-1 0,14-1 0,-10-1 0,40 2 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="3562">1 703 24575,'12'0'0,"37"6"0,11 1 0,38-4 0,-27 2 0,16 1 0,4 1 0,-10-1-2201,11-2 1,8 0 2200,-32-2 0,13 1 0,10 1 0,6-1 0,1 0 0,-2 1 0,-6-1 0,-10 0 0,17 1 0,-12-1 0,1 1 0,11-1 0,-16-1 0,10 0 0,6 0 0,2 0 0,0 0 0,-3-1 0,-7 1 0,-10-1 0,10 1 0,-9 0 0,-4-1 0,-1-1 0,20 0 0,-3-1 0,-7-2 0,1-1 0,-13-3 1350,4-12-1350,-1 0 717,-20-1-717,12 1 0,2 1 0,8-1 0,-9 4 0,6 1-333,12-1 0,12-1 1,4 1 332,-10 5 0,5 1 0,2 1 0,-2-1 0,-3 0 0,-1 0 0,1-1 0,-1 2 551,5 0 0,1 0 0,-3 1 1,-10 1-552,20-4 0,-19 3 0,-18 3 0,-40 6 0,-29 0 0,-2 0 281,-1 0 1,-1-2 0,2 0 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="4647">5403 794 24575,'-20'-5'0,"-14"2"0,-16 3 0,-39 4 0,23 1 0,-10 1-785,2 1 0,-7 1 0,-6-1 785,1-1 0,-4-2 0,-6 1 0,-4-1 0,13 0 0,-5 0 0,-4 1 0,0-2 0,3 1 0,5-1 0,3-1 0,5-1 0,2 0 0,-1 0 0,-1 1 0,-12-1 0,-5 1 0,2 0 0,8 1 0,15-1 0,4 0 0,10 0 281,-4 1 0,9 2-281,19 5 0,-2-3 0,-2 8 0,-39 2 0,-22 1 0,17-6 0,-5 0 0,-7-1 0,19-3 0,-5-1 0,-3 0 0,0 0 0,4-1 260,-9 0 1,3 0 0,0-1-1,-1-2-260,-6-2 0,-3-1 0,3-1 0,10 1 0,-17 0 0,5 0 0,9 0 0,-2 0 0,8 0 0,9-2 0,7 0 0,6 1 0,4 0 0,-10-3 0,21 4 0,-16 4 0,11-3 0,4 5 751,34-4-751,3 0 0,4 0 0,0-2 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="6035">364 1372 20584,'13'-2'0,"15"2"1712,60-7-1712,-29 6 0,2 1 0,23 0 0,13 1 0,2 2 0,-8 0-806,1 3 0,-4 2 0,5 1 1,12 1 805,-22-3 0,9 1 0,7 1 0,5 0 0,3 0 0,-1 1 0,-1 0 0,-3 1 0,-7-1-299,4 2 1,-4 1 0,-3-1 0,-1 2 0,1-1 0,2 1 0,5 0 298,-13-1 0,4 0 0,3 0 0,2 1 0,0 0 0,0 0 0,-3 0 0,-4-1 0,-5 0 0,-6-2 0,17 4 0,-9-2 0,-5 0 0,0-1 0,5 1 0,1 0 0,4 1 0,3 1 0,-3-2 0,-6-3 0,-10-2 126,6-5 0,-10-5 0,0 2-126,2 3 0,0 0 0,-4-2 32,12-5 0,-5-5-32,-4-6 0,-5-2 0,21 3 1280,-10-5 1,6 0-1281,-1 7 0,2 2 0,-19-1 0,3-1 0,0 0 0,6 1 0,1-1 0,0 2 0,-2 3 0,0 0 0,-6-1 2037,-8-4 0,-1-2-2037,39-2 0,-5-2 512,-10-12-512,-19 9 0,-1 1 0,12-12 0,-37 14 0,19-10 0,-23 15 0,16-2 0,-11 8 0,16-3 0,-22 6 0,16-3 0,-3-3 0,-10 1 0,-8 2 0,-24 3 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="6917">7899 1748 24575,'-2'3'0,"-8"8"0,-58 32 0,3-5 0,-13 4 0,15-13 0,-9 0 0,-4 0 0,-5-1 0,1-3 0,-5-1 0,-3 0 0,-4-3 0,-4 0-646,13-5 0,-4 0 1,-3-2-1,-2-1 0,-1 0 1,-1-1-1,-1-1 646,5-1 0,0-1 0,0-1 0,-2-1 0,-2 0 0,-1 0 0,-4 0 0,-2 1-384,15-2 1,-4 1 0,-3-1-1,-3 1 1,-1 0 0,-1 0-1,0-1 1,1 1 0,2-1-1,2 0 1,4-1 0,3 1 383,-12-1 0,5 1 0,3-2 0,1 1 0,2-1 0,-1 1 0,-2-1 0,-4 1 0,-3 0 0,-6 1 0,-4 0 0,0 0 0,1 0 0,3 0 0,8-1 0,8 0 0,12-2 0,-23 2 0,18-1 0,1-2 0,-2-2 0,1-2 0,15 1 0,-1 0 0,8-3 0,-8 1 0,-28 2 0,-9 1 0,23-1 0,-4-1 0,-8 0 137,8 1 1,-9-1 0,-3-1 0,3 1-1,7 0-137,-13 0 0,7 0 0,-1-1 0,14 1 0,-3-1 0,5 0 0,15 0 5968,-21-4-5968,69 5 0,10-4 0,0 2 0,-1-2 0,2 5 0,3 0 0,0 3 0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink35.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-07-26T07:43:12.302"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">470 699 24575,'4'0'0,"60"1"0,-10 3 0,3-2 0,11 2 0,7 8 0,8 4 0,8 0 0,-14-4 0,5 0 0,5 1 0,1 0 0,2 0-1639,-7-1 1,3 1-1,1 0 1,1 1 0,0-2-1,-1 1 1390,-3-1 1,-1-1 0,0 0 0,0 0-1,0 0 1,0-1 248,16 2 0,0 1 0,-1-2 0,-1 0 0,-2-1 221,-10-2 0,-2-1 0,-1-1 0,-1 0 0,-3 1-221,7 1 0,-4 2 0,0-1 0,2-1 232,14-1 1,5-1 0,-4-2 0,-12 1-233,5 1 0,-3-1 0,-2-1 0,6-1 0,-5 1 0,2-1 0,1 0 0,-3-2 0,8-1 0,-2-2 0,-8-1 0,0-1 0,0-1-164,1 1 1,0 0 0,4-1 163,-6 0 0,4 0 0,-1-1 0,-8 0 0,14-3 0,6 0 0,-29 4 0,10 0 0,7 1 0,3-1 0,-1 0 0,-4-1 335,6-1 1,-3 0 0,0-1-1,4 0 1,6 1-336,-15 2 0,4 0 0,3 0 0,3 0 0,1 0 0,1 0 0,-1 0 0,-2 0 0,-1-1 0,2 1 0,-1-1 0,1 0 0,-1 0 0,-1 0 0,-1 1 0,-2-1 0,2 0 0,-2 0 0,-2-1 0,0 1 0,0 0 0,0 0 0,1 1 0,3-1 0,-2 1 0,1 0 0,1 0 0,1 0 0,3-1 0,2-1 0,-6 1 0,4-2 0,2 0 0,2 0 0,0-1 0,0 0 0,-1 1 0,-2 0 0,-2 0-411,7 1 1,-5 0 0,-2 0 0,0 0 0,3 0 0,7 0 0,10-2 410,-32 3 0,5 0 0,5-1 0,4-1 0,4 0 0,2 1 0,3-1 0,0-1 0,0 1 0,0 0 0,-1 0 0,-2 1 0,-4-1 0,-3 1 0,-4 0 0,-6 1 0,17-1 0,-5 0 0,-6 1 0,-3 0 0,-1 0 0,0 0 0,2 0 0,4 0 0,5 0 0,-11 0 0,4-1 0,3 1 0,1-1 0,2 1 0,2-1 0,-1 0 0,1 0 0,-1 1 0,-2-1 0,-2 1 0,-2 0 0,-4 0-287,17 0 0,-4 0 0,-1 0 1,-2 1-1,-2 0 0,0 0 0,-2-1 1,0 1-1,0 0 287,4-1 0,-1 0 0,-1 0 0,-1 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-2 0 0,-1 0 0,0 0 0,0 0 0,0 0 0,-2 1 0,-1-1 0,-2 0-120,19-2 0,1 1 1,-1-1-1,-5 0 1,-7 1-1,-8 1 120,8-1 0,-11 0 0,2 1 606,11-3 0,2 1 0,-10-1-606,-8-1 0,-8 1 0,-12 1 0,5 0 0,2 1 0,10-1 0,6 0 0,-1 1 497,6 1 1,2 0 0,2 0-1,3-1-497,-4 0 0,3 0 0,3-1 0,-2 1 0,-3-1 0,7 1 0,-3-1 0,-1 1 0,-2-1 0,-7 1 0,-2-1 0,-1 1 0,-1 0 1437,20 0 0,-1 1 1,1 1-1438,-15 2 0,2 0 0,0 0 0,-2 1 0,15-1 0,-1 2 0,-3 0 0,-6 2 0,-1 0 0,-9 1 0,-6 1 0,0 0 0,-1 0 0,7 1 0,0 0 0,-6 1 0,0 1 0,6-1 0,4-1 0,8-2 0,0 1 0,-7 1 0,-2 2 0,-5 2 0,6 0 0,-9-2 0,5 0 0,4 0 0,0 1 0,-4 1 0,11 2 0,-3 1 0,1 0 0,2-1 0,-5-1 0,3 0 0,2 0 0,-2-1 0,-3 0 0,8 1 0,-3 1 0,-1-2 0,-2-1 0,-4-2 0,1-2 0,-5-1 0,-13 0 0,-6 1 0,-6-1 1194,15-2 1,-15 0-1195,-40 4 0,20 7 0,53 13 0,-9-7 0,7 1 0,-5-2 0,6 1 0,3 1 0,9 1 0,0-2 0,0-5 0,0-2 0,-4 1 0,-12 2 0,-2 1 0,-4-2 0,-4-5 0,-2-2 0,-14-1 0,-6 0 2867,-41-2-2867,18-4 891,-18 1-891,7-1 0,0 0 0,-12 2 0,7 0 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1249">26537 871 15357,'-71'13'0,"-7"1"0,-15 4 0,25-6 0,-4 0 0,-6 2 0,-7 0 0,3 0 0,-7 1 0,-5 0 0,-3 0 0,-2 0 0,1-1-440,6-2 0,1-1 0,-1-1 1,-2 0-1,-4 0 0,-4 0 1,-5 1 439,25-3 0,-4 1 0,-5 0 0,-2 0 0,-2 1 0,-2-1 0,-1 0 0,0 1 0,1-1 0,0-1 0,3 0 0,2 0 0,3-1-112,-9 1 0,3-2 0,2 0 0,2 0 1,0-1-1,1 0 0,-1 1 0,-1-1 1,-2 0-1,-1 1 112,5 0 0,-4 0 0,-2 1 0,-2-1 0,0 1 0,0 0 0,1-1 0,2 0 0,3 0 0,5-1 0,4 0 0,7-1 0,-33 1 0,11-1 0,6 0 0,3-1 0,-3 0 0,0 1 0,-2 1 0,1 0 0,6-2 0,7-2 488,-1-4 0,9-2 1,-7 0-489,-7 2 0,-8 0 0,-1 0 0,4-2 0,14-2 0,3-2 0,1 0 0,-3 1 0,-7 1 0,-2 1 0,-2 0 0,-2 0 47,7 1 1,-2 0 0,-3 0 0,-1 0 0,-1 1-48,4 1 0,-1 1 0,-2 0 0,-1 0 0,-2 0 0,-2 0 40,1 1 0,-3-1 0,-3 1 1,0-1-1,0 1 0,1 0 1,3 0-41,-6 1 0,3 0 0,0 0 0,0 0 0,-2 0 0,-4 0 0,10 0 0,-3 1 0,-2-1 0,-2 0 0,0 0 0,1 0 0,2 1 0,3-1-79,1 0 0,1 0 0,2 0 1,1 0-1,0 0 0,1 0 0,0 0 79,-12-1 0,2 1 0,-1-1 0,1 1 0,-2 0 0,-1 0 0,3 1 0,-3 0 0,-2 1 0,1-1 0,1 1 0,5 0 0,6 0-94,3 1 1,7-1 0,2 1-1,-3 0 1,-8 1 93,6-1 0,-7 1 0,-4-1 0,-2 1 0,-3 0 0,2 0 0,2 0 0,3 0 0,1-1 0,3 1 0,0 0 0,1 0 0,1-1 0,-2 1 0,-1-1-257,-5 0 0,0 0 1,0 0-1,-1 0 0,-2 0 1,-2 0-1,-4 0 257,15 0 0,-2 0 0,-2 0 0,-2-1 0,-1 2 0,-1-1 0,-1 0 0,0 0 0,1-1 0,-1 1 0,7 0 0,0-1 0,0 1 0,0-1 0,-1 1 0,0-1 0,0 1 0,-2-1 0,0 1 0,-1-1 0,-1 1 0,5 0 0,-1-1 0,-1 1 0,-2-1 0,0 1 0,0 0 0,-1-1 0,0 1 0,1 0 0,0-1 0,0 1 0,2 0 0,0-1 0,-11 1 0,0 1 0,-1-1 0,1 0 0,0 0 0,1 0 0,1 0 0,3 0 0,2 0 0,3 0 0,3-1 0,-17 1 0,3 0 0,3 0 0,4-1 0,3 1 0,3-1 0,3 0 0,-6 1 0,5 1 0,4-1 0,2-1 0,1-1 0,-3-1 0,3-2 0,0 0 0,-2 1 292,-8 0 0,-2 0 0,-2 1 1,-6 0-293,14 1 0,-4 1 0,-3 0 0,-2 0 0,1 0 0,1 0 0,3-1 0,-1 0 0,1 0 0,0 1 0,0-1 0,1 2 382,-1 1 0,1 1 0,0 0 0,0 0 1,0 0-1,2-1-382,2-1 0,0-1 0,0 0 0,2 0 0,3 0 0,5 1 0,-7 1 0,6 1 0,1-1 0,-5-1 0,0-1 0,-6-1 0,-1 0 0,4-2 0,7 0 176,-6-2 0,8-1 1,-10-1-177,10 0 0,-9-1 0,-4-1 0,-3-1 0,0 1 0,4-1 0,-9-2 0,4 1 0,-2-1 0,-3-1 0,-8-1 152,20 3 0,-7-2 0,-6 0 1,-3-1-1,0 0 0,2 0 1,4 1-1,6 0 0,9 2-152,-24-4 0,11 3 0,5-1 0,-7-1 0,-5-1 0,-14-1 0,4-1 0,21 3 0,37 4 0,39 4 0,14 2 0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink36.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-07-26T07:43:15.684"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.025" units="cm"/>
+      <inkml:brushProperty name="height" value="0.025" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">443 255 11241,'16'0'0,"24"0"-348,21 3 1,30 3 0,14 1 0,-1 0 0,-16-2 347,-13-3 0,-9 0 0,17 1 0,-16-1 0,11 1 0,8 1 0,7 1 0,5-1 0,4 0 0,0 1 0,0-2 0,-3 1 0,-4-2-48,-5 0 0,-2-1 0,-2-1 0,0 0 0,0 0 0,2 0 1,3 0-1,4-1 0,3 1 0,7 0 48,-22 0 0,4 0 0,3 0 0,2 0 0,3 0 0,3 0 0,1 0 0,2 0 0,1 0 0,2 0 0,0 0 0,1-1 0,0 1 0,0 0 0,0 0 0,-2 0 0,0-1 0,-1 1 0,-2 0-12,-1-1 0,-1 1 0,0 0 1,0-1-1,-1 1 0,1-1 0,-1 0 1,0 1-1,1-1 0,0 1 0,0-1 1,1 0-1,0 1 0,1-1 1,1 1-1,1-1 0,0 0 0,2 1 1,2-1 11,-14 1 0,3-1 0,0 1 0,3-1 0,0 1 0,2-1 0,0 1 0,1-1 0,1 1 0,0-1 0,1 1 0,-1-1 0,1 1 0,-1 0 0,-1-1 0,0 0 0,0 1 0,-2-1 0,0 1 0,-2-1 0,-2 1 0,-1-1 0,-1 1 0,-3-1 0,-2 0-39,20 1 1,-3-1 0,-4 0 0,-1 0-1,-2 0 1,-2-1 0,-1 1 0,0 0 0,-1 0-1,0 0 1,1 0 0,0 0 0,2 0 0,1 1-1,3-1 1,2 0 38,-8 1 0,2 0 0,3-1 0,1 1 0,1 0 0,2 0 0,0 1 0,1-1 0,1 0 0,-1 0 0,-1 0 0,0 0 0,-1 0 0,-2 0 0,-1 0 0,-2 0 0,-2 0 0,-3 0 0,-2-1 0,-4 1 0,18-2 0,-4 1 0,-4 0 0,-2-1 0,-3 1 0,-2-1 0,0 0 0,0 0 0,-1 1 0,2-1 0,1 1 0,3-1 0,-2 1 0,4 0 0,1 0 0,1 0 0,1 0 0,0 0 0,-1 0 0,-2 0 0,-2 0 0,-2 0 0,-4 0 0,-4 0 0,-4 0 138,17-1 1,-5 0 0,-6 0 0,-2 0 0,-4 0 0,0 0 0,0 0-139,18-1 0,-3 1 0,-2 0 0,-1 0 0,2 0 292,1 0 0,-2 1 0,1 0 0,3 0 0,2 0-292,-15 1 0,3 0 0,1 0 0,1 0 0,1-1 0,0 1 0,-2 0 0,-1-1 0,-1 1 0,1-1 0,-1 0 0,0 0 0,-1 0 0,1 1 201,11-1 1,2 1-1,-2 1 1,0-1-1,-3 0 1,-3 0-202,-1-1 0,-4 0 0,-1 0 0,-2 0 0,0-1 0,16 0 0,0-1 0,-5 1 0,-8-1 908,-11 1 0,-7-1 1,-6 0-909,13-3 0,-24 1 2181,-44 5-2181,85-7 0,-21 2 0,13-1 0,9 0 0,-10 2 0,6 0 0,5 0 0,4 0 0,1-1-404,-17 0 0,4 0 0,2 0 1,1-1-1,-1 0 0,-2 1 1,-3 0 403,13 1 0,-3-1 0,-2 2 0,0-2 0,1 0 0,10-1 0,6-2 0,-2 1 0,-10-1 0,-20 3 1284,-12 0 0,-8 1-1284,41-6 0,-25 2 1311,-64 8-1311,-3-4 0,-1 2 0,1-2 6784,-3 0-6784,2 1 0,-1 5 0,0-1 0,-2 3 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="995">22348 222 24575,'-66'24'0,"3"-8"0,-24 5 0,-17 2 0,-7 0 0,1 0 0,8-4 0,15-4 0,3-2 0,1-1 0,-3-1 0,-3 2 0,-8 1-984,12 0 1,-3 1 0,-3 1 0,-3 1 0,-4 0 0,-1 0 0,-3 0 0,-2-1 0,-2-1 0,-1-2 883,18-3 1,-1-1 0,-2-1-1,-1 0 1,-1 0 0,-2-1-1,-1-1 1,-1 1 0,-2-2 0,-2 1-1,0-1 1,-2 1 0,-2-1-1,-1-1 1,-1 1 5,19-1 0,-1-1 1,-3 0-1,-2 0 0,-1 0 1,-2-1-1,-1 0 0,0 0 1,-2 0-1,0 0 0,-1-1 1,0 1-1,-1 0 0,1-1 1,1 0-1,-1 1 0,2-1 1,0 1-1,1 0 0,1 0 1,2 0-1,2 0 0,1 0 94,-10 1 0,4 0 0,1 0 0,2 0 0,1 1 0,2-1 0,0 0 0,0 1 0,1-1 0,-1 1 0,-1-1 0,-1 0 0,-1 0 0,-2 0 0,-3 0 0,-2 0 0,-3-1 0,-3 0-29,23-1 1,-3 1-1,-2-1 1,-3 0 0,-1 0-1,-2 0 1,-2-1 0,-1 1-1,-2 0 1,0-1 0,-2 0-1,0 1 1,-1-1 0,-1 0-1,1 0 1,-1 0 0,1 0-1,0 0 1,0 0 0,1 0-1,1 0 1,1 0 0,2 0-1,0 0 1,3 0 0,1 0-1,2 0 1,2 0 0,2 1-1,3-1 1,3 0 28,-24 0 0,3 0 0,4 0 0,3 1 0,2-1 0,2 0 0,2 0 0,1 0 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,-2-1 0,-1 0 0,-3 0 0,-2 1-97,6-1 0,-1 0 1,-1 1-1,-2-1 1,-2 1-1,0-1 0,-1 1 1,0 0-1,-1-1 1,0 1-1,0-1 1,1 1-1,0 0 0,1-1 1,1 1-1,1-1 1,1 1-1,2-1 0,2 1 1,2-1-1,3 0 97,-17 1 0,1-1 0,3 0 0,0 0 0,2 1 0,1-1 0,2 0 0,1 0 0,2 0 0,1 0 0,2-1 0,1 1 0,1 0 0,1-1 0,-20 0 0,0 0 0,1 0 0,3-1 0,3 1 0,3-1 0,5 1 0,4 0 0,7 0 0,-25 0 0,12 0 0,4 1 0,-8-1 271,13-1 0,-5 0 1,-3-1-1,0 1 1,1 0-1,2 1-271,-9 2 0,1 2 0,2 0 0,0 0 0,3-1 0,10 0 0,2-1 0,2 1 0,-2 0 0,-3-1 320,-1 1 0,-4 0 0,-2 1 1,2-1-1,4 0 0,7 1-320,-21 0 0,9 0 0,-1 1 0,15-2 0,0 0 0,-2 1 0,2 1 0,-23 3 0,2 1 0,-5 0 0,10-3 0,-4-1 0,0 1 0,5 0 0,-7 2 0,4 1 0,-6-1 0,14-3 0,-6-2 0,-2 0 0,0 0 0,4 0 603,-5 1 0,4 0 0,0 0 1,-2 0-604,9-2 0,-1 1 0,-2-1 0,3 0 0,4 0-716,-3 1 1,1-1 0,6 0 0,9 0 715,-7 0 0,7-2 430,3-2 1,5-1-431,-11 3 997,5-6 1,25 7 0,34 0 0</inkml:trace>
+</inkml:ink>
+</file>
+
 <file path=xl/ink/ink4.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
@@ -10110,11 +10553,11 @@
       <c r="E6" t="s">
         <v>505</v>
       </c>
-      <c r="G6" s="76" t="s">
+      <c r="G6" s="83" t="s">
         <v>515</v>
       </c>
-      <c r="H6" s="76"/>
-      <c r="I6" s="76"/>
+      <c r="H6" s="83"/>
+      <c r="I6" s="83"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
       <c r="G7" t="s">
@@ -10220,12 +10663,12 @@
       <c r="E23" t="s">
         <v>526</v>
       </c>
-      <c r="G23" s="76" t="s">
+      <c r="G23" s="83" t="s">
         <v>525</v>
       </c>
-      <c r="H23" s="76"/>
-      <c r="I23" s="76"/>
-      <c r="J23" s="76"/>
+      <c r="H23" s="83"/>
+      <c r="I23" s="83"/>
+      <c r="J23" s="83"/>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.2">
       <c r="C24" t="s">
@@ -10253,10 +10696,10 @@
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="G26" s="76" t="s">
+      <c r="G26" s="83" t="s">
         <v>529</v>
       </c>
-      <c r="H26" s="76"/>
+      <c r="H26" s="83"/>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.2">
       <c r="D30" t="s">
@@ -11579,7 +12022,7 @@
       <c r="D84">
         <v>1</v>
       </c>
-      <c r="E84" s="76">
+      <c r="E84" s="83">
         <v>20</v>
       </c>
       <c r="F84">
@@ -11602,7 +12045,7 @@
       <c r="D85">
         <v>2</v>
       </c>
-      <c r="E85" s="76"/>
+      <c r="E85" s="83"/>
       <c r="F85">
         <v>2</v>
       </c>
@@ -11623,7 +12066,7 @@
       <c r="D86">
         <v>3</v>
       </c>
-      <c r="E86" s="76">
+      <c r="E86" s="83">
         <v>20</v>
       </c>
       <c r="F86">
@@ -11643,7 +12086,7 @@
       <c r="D87">
         <v>4</v>
       </c>
-      <c r="E87" s="76"/>
+      <c r="E87" s="83"/>
     </row>
     <row r="88" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C88">
@@ -11652,7 +12095,7 @@
       <c r="D88">
         <v>5</v>
       </c>
-      <c r="E88" s="76">
+      <c r="E88" s="83">
         <v>20</v>
       </c>
     </row>
@@ -11663,7 +12106,7 @@
       <c r="D89">
         <v>6</v>
       </c>
-      <c r="E89" s="76"/>
+      <c r="E89" s="83"/>
     </row>
     <row r="90" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C90">
@@ -11672,7 +12115,7 @@
       <c r="D90">
         <v>7</v>
       </c>
-      <c r="E90" s="76">
+      <c r="E90" s="83">
         <v>20</v>
       </c>
     </row>
@@ -11683,7 +12126,7 @@
       <c r="D91">
         <v>8</v>
       </c>
-      <c r="E91" s="76"/>
+      <c r="E91" s="83"/>
     </row>
     <row r="92" spans="3:9" x14ac:dyDescent="0.2">
       <c r="C92">
@@ -11692,7 +12135,7 @@
       <c r="D92">
         <v>9</v>
       </c>
-      <c r="E92" s="76">
+      <c r="E92" s="83">
         <v>20</v>
       </c>
     </row>
@@ -11703,7 +12146,7 @@
       <c r="D93">
         <v>10</v>
       </c>
-      <c r="E93" s="76"/>
+      <c r="E93" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -26126,7 +26569,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C5EE1AE-2986-774A-BCF0-09073C7E34EA}">
-  <dimension ref="B2:K115"/>
+  <dimension ref="B2:K181"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
@@ -26155,7 +26598,7 @@
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="G4" s="77" t="s">
+      <c r="G4" s="71" t="s">
         <v>625</v>
       </c>
     </row>
@@ -26302,136 +26745,136 @@
       </c>
     </row>
     <row r="41" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B41" s="79"/>
+      <c r="B41" s="72"/>
       <c r="C41" s="33"/>
       <c r="D41" s="33"/>
       <c r="E41" s="34"/>
-      <c r="H41" s="79"/>
+      <c r="H41" s="72"/>
       <c r="J41" t="s">
         <v>652</v>
       </c>
     </row>
     <row r="42" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B42" s="80"/>
-      <c r="C42" s="78"/>
-      <c r="D42" s="78"/>
+      <c r="B42" s="73"/>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
       <c r="E42" s="36"/>
-      <c r="H42" s="80"/>
+      <c r="H42" s="73"/>
     </row>
     <row r="43" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B43" s="80"/>
-      <c r="C43" s="78"/>
-      <c r="D43" s="78"/>
+      <c r="B43" s="73"/>
+      <c r="C43" s="6"/>
+      <c r="D43" s="6"/>
       <c r="E43" s="36"/>
-      <c r="H43" s="80"/>
+      <c r="H43" s="73"/>
       <c r="J43" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="44" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B44" s="80"/>
-      <c r="C44" s="78"/>
-      <c r="D44" s="78"/>
+      <c r="B44" s="73"/>
+      <c r="C44" s="6"/>
+      <c r="D44" s="6"/>
       <c r="E44" s="36"/>
-      <c r="H44" s="80"/>
+      <c r="H44" s="73"/>
     </row>
     <row r="45" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B45" s="80"/>
-      <c r="C45" s="78"/>
-      <c r="D45" s="78"/>
+      <c r="B45" s="73"/>
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
       <c r="E45" s="36"/>
-      <c r="H45" s="80"/>
+      <c r="H45" s="73"/>
     </row>
     <row r="46" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B46" s="80"/>
-      <c r="C46" s="78"/>
-      <c r="D46" s="78"/>
+      <c r="B46" s="73"/>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
       <c r="E46" s="36"/>
-      <c r="H46" s="80"/>
+      <c r="H46" s="73"/>
     </row>
     <row r="47" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B47" s="80"/>
-      <c r="C47" s="78"/>
-      <c r="D47" s="78"/>
+      <c r="B47" s="73"/>
+      <c r="C47" s="6"/>
+      <c r="D47" s="6"/>
       <c r="E47" s="36"/>
-      <c r="H47" s="80"/>
+      <c r="H47" s="73"/>
     </row>
     <row r="48" spans="2:10" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="80"/>
-      <c r="C48" s="78"/>
-      <c r="D48" s="78"/>
+      <c r="B48" s="73"/>
+      <c r="C48" s="6"/>
+      <c r="D48" s="6"/>
       <c r="E48" s="36"/>
-      <c r="H48" s="80"/>
+      <c r="H48" s="73"/>
     </row>
     <row r="49" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B49" s="79"/>
+      <c r="B49" s="72"/>
       <c r="C49" s="33"/>
       <c r="D49" s="33"/>
       <c r="E49" s="34"/>
-      <c r="H49" s="82"/>
+      <c r="H49" s="75"/>
     </row>
     <row r="50" spans="2:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="81"/>
+      <c r="B50" s="74"/>
       <c r="C50" s="38"/>
       <c r="D50" s="38"/>
       <c r="E50" s="39"/>
-      <c r="H50" s="83"/>
+      <c r="H50" s="76"/>
     </row>
     <row r="51" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B51" s="80"/>
-      <c r="C51" s="78"/>
-      <c r="D51" s="78"/>
+      <c r="B51" s="73"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="6"/>
       <c r="E51" s="36"/>
-      <c r="H51" s="80"/>
+      <c r="H51" s="73"/>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B52" s="80"/>
-      <c r="C52" s="78"/>
-      <c r="D52" s="78"/>
+      <c r="B52" s="73"/>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
       <c r="E52" s="36"/>
-      <c r="H52" s="80"/>
+      <c r="H52" s="73"/>
     </row>
     <row r="53" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B53" s="80"/>
-      <c r="C53" s="78"/>
-      <c r="D53" s="78"/>
+      <c r="B53" s="73"/>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
       <c r="E53" s="36"/>
-      <c r="H53" s="80"/>
+      <c r="H53" s="73"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B54" s="80"/>
-      <c r="C54" s="78"/>
-      <c r="D54" s="78"/>
+      <c r="B54" s="73"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
       <c r="E54" s="36"/>
-      <c r="H54" s="80"/>
+      <c r="H54" s="73"/>
     </row>
     <row r="55" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B55" s="80"/>
-      <c r="C55" s="78"/>
-      <c r="D55" s="78"/>
+      <c r="B55" s="73"/>
+      <c r="C55" s="6"/>
+      <c r="D55" s="6"/>
       <c r="E55" s="36"/>
-      <c r="H55" s="80"/>
+      <c r="H55" s="73"/>
     </row>
     <row r="56" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B56" s="80"/>
-      <c r="C56" s="78"/>
-      <c r="D56" s="78"/>
+      <c r="B56" s="73"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
       <c r="E56" s="36"/>
-      <c r="H56" s="80"/>
+      <c r="H56" s="73"/>
     </row>
     <row r="57" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B57" s="80"/>
-      <c r="C57" s="78"/>
-      <c r="D57" s="78"/>
+      <c r="B57" s="73"/>
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
       <c r="E57" s="36"/>
-      <c r="H57" s="80"/>
+      <c r="H57" s="73"/>
     </row>
     <row r="58" spans="2:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="81"/>
+      <c r="B58" s="74"/>
       <c r="C58" s="38"/>
       <c r="D58" s="38"/>
       <c r="E58" s="39"/>
-      <c r="H58" s="81"/>
+      <c r="H58" s="74"/>
     </row>
     <row r="63" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B63" s="7"/>
@@ -26452,20 +26895,20 @@
       <c r="E68" s="7"/>
     </row>
     <row r="69" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B69" s="84"/>
-      <c r="E69" s="84"/>
+      <c r="B69" s="77"/>
+      <c r="E69" s="77"/>
     </row>
     <row r="70" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B70" s="84"/>
+      <c r="B70" s="77"/>
     </row>
     <row r="71" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B71" s="84"/>
+      <c r="B71" s="77"/>
     </row>
     <row r="72" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B72" s="84"/>
+      <c r="B72" s="77"/>
     </row>
     <row r="73" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B73" s="84"/>
+      <c r="B73" s="77"/>
     </row>
     <row r="76" spans="2:11" x14ac:dyDescent="0.2">
       <c r="C76" t="s">
@@ -26646,20 +27089,14 @@
     </row>
     <row r="100" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B100" s="26"/>
-      <c r="C100" s="85"/>
-      <c r="D100" s="85"/>
       <c r="E100" s="27"/>
     </row>
     <row r="101" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B101" s="26"/>
-      <c r="C101" s="85"/>
-      <c r="D101" s="85"/>
       <c r="E101" s="27"/>
     </row>
     <row r="102" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B102" s="26"/>
-      <c r="C102" s="85"/>
-      <c r="D102" s="85"/>
       <c r="E102" s="27"/>
       <c r="G102" s="23" t="s">
         <v>662</v>
@@ -26670,8 +27107,6 @@
     </row>
     <row r="103" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B103" s="26"/>
-      <c r="C103" s="85"/>
-      <c r="D103" s="85"/>
       <c r="E103" s="27"/>
       <c r="G103" s="26" t="s">
         <v>663</v>
@@ -26682,8 +27117,6 @@
     </row>
     <row r="104" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B104" s="26"/>
-      <c r="C104" s="85"/>
-      <c r="D104" s="85"/>
       <c r="E104" s="27"/>
       <c r="G104" s="28" t="s">
         <v>664</v>
@@ -26694,8 +27127,6 @@
     </row>
     <row r="105" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B105" s="26"/>
-      <c r="C105" s="85"/>
-      <c r="D105" s="85"/>
       <c r="E105" s="27"/>
     </row>
     <row r="106" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -26740,14 +27171,10 @@
     </row>
     <row r="110" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B110" s="26"/>
-      <c r="C110" s="85"/>
-      <c r="D110" s="85"/>
       <c r="E110" s="27"/>
     </row>
     <row r="111" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B111" s="26"/>
-      <c r="C111" s="85"/>
-      <c r="D111" s="85"/>
       <c r="E111" s="27"/>
       <c r="G111" s="23" t="s">
         <v>662</v>
@@ -26758,8 +27185,6 @@
     </row>
     <row r="112" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B112" s="26"/>
-      <c r="C112" s="85"/>
-      <c r="D112" s="85"/>
       <c r="E112" s="27"/>
       <c r="G112" s="26" t="s">
         <v>663</v>
@@ -26768,10 +27193,8 @@
         <v>20</v>
       </c>
     </row>
-    <row r="113" spans="2:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B113" s="26"/>
-      <c r="C113" s="85"/>
-      <c r="D113" s="85"/>
       <c r="E113" s="27"/>
       <c r="G113" s="28" t="s">
         <v>665</v>
@@ -26780,20 +27203,86 @@
         <v>40</v>
       </c>
     </row>
-    <row r="114" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B114" s="26"/>
-      <c r="C114" s="85"/>
-      <c r="D114" s="85"/>
       <c r="E114" s="27"/>
     </row>
-    <row r="115" spans="2:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B115" s="28"/>
       <c r="C115" s="9"/>
       <c r="D115" s="9"/>
       <c r="E115" s="29"/>
     </row>
+    <row r="123" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="J123" t="s">
+        <v>444</v>
+      </c>
+      <c r="K123">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="126" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="J126" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="129" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="10:10" x14ac:dyDescent="0.2">
+      <c r="J130">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B173" s="64"/>
+      <c r="D173" s="84"/>
+      <c r="E173" s="84"/>
+      <c r="F173" s="84"/>
+      <c r="G173" s="84"/>
+      <c r="H173" s="84"/>
+      <c r="I173" s="84"/>
+      <c r="J173" s="84"/>
+      <c r="K173" s="84"/>
+    </row>
+    <row r="174" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B174" s="65"/>
+    </row>
+    <row r="175" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B175" s="65"/>
+    </row>
+    <row r="176" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B176" s="65"/>
+    </row>
+    <row r="177" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B177" s="65"/>
+    </row>
+    <row r="178" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B178" s="65"/>
+    </row>
+    <row r="179" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B179" s="65"/>
+    </row>
+    <row r="180" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B180" s="65"/>
+    </row>
+    <row r="181" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B181" s="66"/>
+      <c r="D181" s="84"/>
+      <c r="E181" s="84"/>
+      <c r="F181" s="84"/>
+      <c r="G181" s="84"/>
+      <c r="H181" s="84"/>
+      <c r="I181" s="84"/>
+      <c r="J181" s="84"/>
+      <c r="K181" s="84"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -26954,7 +27443,7 @@
     <row r="20" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C20" s="5">
         <f ca="1">NOW()</f>
-        <v>46228.910883680554</v>
+        <v>46229.550143518522</v>
       </c>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.2">
@@ -27614,29 +28103,29 @@
       <c r="B102" t="s">
         <v>90</v>
       </c>
-      <c r="I102" s="71" t="s">
+      <c r="I102" s="78" t="s">
         <v>101</v>
       </c>
-      <c r="J102" s="71"/>
-      <c r="K102" s="71"/>
+      <c r="J102" s="78"/>
+      <c r="K102" s="78"/>
     </row>
     <row r="103" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B103" t="s">
         <v>102</v>
       </c>
-      <c r="I103" s="71"/>
-      <c r="J103" s="71"/>
-      <c r="K103" s="71"/>
+      <c r="I103" s="78"/>
+      <c r="J103" s="78"/>
+      <c r="K103" s="78"/>
     </row>
     <row r="104" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="I104" s="71"/>
-      <c r="J104" s="71"/>
-      <c r="K104" s="71"/>
+      <c r="I104" s="78"/>
+      <c r="J104" s="78"/>
+      <c r="K104" s="78"/>
     </row>
     <row r="105" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="I105" s="71"/>
-      <c r="J105" s="71"/>
-      <c r="K105" s="71"/>
+      <c r="I105" s="78"/>
+      <c r="J105" s="78"/>
+      <c r="K105" s="78"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -27754,7 +28243,7 @@
       <c r="J11" s="8"/>
       <c r="K11" s="8"/>
       <c r="L11" s="14"/>
-      <c r="N11" s="71" t="s">
+      <c r="N11" s="78" t="s">
         <v>114</v>
       </c>
       <c r="O11" t="s">
@@ -27774,7 +28263,7 @@
       <c r="J12" s="8"/>
       <c r="K12" s="8"/>
       <c r="L12" s="14"/>
-      <c r="N12" s="71"/>
+      <c r="N12" s="78"/>
       <c r="O12" t="s">
         <v>116</v>
       </c>
@@ -27792,7 +28281,7 @@
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
       <c r="L13" s="14"/>
-      <c r="N13" s="71"/>
+      <c r="N13" s="78"/>
       <c r="O13" t="s">
         <v>117</v>
       </c>
@@ -28068,7 +28557,7 @@
       <c r="F48" t="s">
         <v>157</v>
       </c>
-      <c r="H48" s="71" t="s">
+      <c r="H48" s="78" t="s">
         <v>160</v>
       </c>
     </row>
@@ -28076,13 +28565,13 @@
       <c r="F49" t="s">
         <v>158</v>
       </c>
-      <c r="H49" s="71"/>
+      <c r="H49" s="78"/>
     </row>
     <row r="50" spans="4:10" x14ac:dyDescent="0.2">
       <c r="F50" t="s">
         <v>159</v>
       </c>
-      <c r="H50" s="71"/>
+      <c r="H50" s="78"/>
     </row>
     <row r="52" spans="4:10" x14ac:dyDescent="0.2">
       <c r="D52" t="s">
@@ -30036,34 +30525,34 @@
       </c>
     </row>
     <row r="170" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C170" s="71" t="s">
+      <c r="C170" s="78" t="s">
         <v>376</v>
       </c>
-      <c r="D170" s="71"/>
-      <c r="E170" s="71"/>
-      <c r="F170" s="71"/>
-      <c r="G170" s="71"/>
+      <c r="D170" s="78"/>
+      <c r="E170" s="78"/>
+      <c r="F170" s="78"/>
+      <c r="G170" s="78"/>
     </row>
     <row r="171" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C171" s="71"/>
-      <c r="D171" s="71"/>
-      <c r="E171" s="71"/>
-      <c r="F171" s="71"/>
-      <c r="G171" s="71"/>
+      <c r="C171" s="78"/>
+      <c r="D171" s="78"/>
+      <c r="E171" s="78"/>
+      <c r="F171" s="78"/>
+      <c r="G171" s="78"/>
     </row>
     <row r="173" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C173" s="71"/>
-      <c r="D173" s="71"/>
-      <c r="E173" s="71"/>
-      <c r="F173" s="71"/>
-      <c r="G173" s="71"/>
+      <c r="C173" s="78"/>
+      <c r="D173" s="78"/>
+      <c r="E173" s="78"/>
+      <c r="F173" s="78"/>
+      <c r="G173" s="78"/>
     </row>
     <row r="174" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="C174" s="71"/>
-      <c r="D174" s="71"/>
-      <c r="E174" s="71"/>
-      <c r="F174" s="71"/>
-      <c r="G174" s="71"/>
+      <c r="C174" s="78"/>
+      <c r="D174" s="78"/>
+      <c r="E174" s="78"/>
+      <c r="F174" s="78"/>
+      <c r="G174" s="78"/>
     </row>
     <row r="175" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C175" t="s">
@@ -30221,13 +30710,13 @@
       </c>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="H8" s="71" t="s">
+      <c r="H8" s="78" t="s">
         <v>399</v>
       </c>
       <c r="I8">
         <v>5</v>
       </c>
-      <c r="K8" s="71" t="s">
+      <c r="K8" s="78" t="s">
         <v>400</v>
       </c>
       <c r="L8">
@@ -30247,12 +30736,12 @@
       <c r="F9">
         <v>50</v>
       </c>
-      <c r="H9" s="71"/>
-      <c r="K9" s="71"/>
+      <c r="H9" s="78"/>
+      <c r="K9" s="78"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="H10" s="71"/>
-      <c r="K10" s="71"/>
+      <c r="H10" s="78"/>
+      <c r="K10" s="78"/>
     </row>
     <row r="11" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
@@ -30267,8 +30756,8 @@
       <c r="F11">
         <v>30</v>
       </c>
-      <c r="H11" s="71"/>
-      <c r="K11" s="71"/>
+      <c r="H11" s="78"/>
+      <c r="K11" s="78"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
@@ -30448,7 +30937,7 @@
     </row>
     <row r="33" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="34" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B34" s="72" t="s">
+      <c r="B34" s="79" t="s">
         <v>415</v>
       </c>
       <c r="D34" s="32"/>
@@ -30462,7 +30951,7 @@
       <c r="L34" s="34"/>
     </row>
     <row r="35" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B35" s="73"/>
+      <c r="B35" s="80"/>
       <c r="D35" s="35"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
@@ -30474,7 +30963,7 @@
       <c r="L35" s="36"/>
     </row>
     <row r="36" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B36" s="73"/>
+      <c r="B36" s="80"/>
       <c r="D36" s="35"/>
       <c r="E36" s="6"/>
       <c r="F36" s="6"/>
@@ -30486,7 +30975,7 @@
       <c r="L36" s="36"/>
     </row>
     <row r="37" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="73"/>
+      <c r="B37" s="80"/>
       <c r="D37" s="35"/>
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
@@ -30498,7 +30987,7 @@
       <c r="L37" s="36"/>
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B38" s="73"/>
+      <c r="B38" s="80"/>
       <c r="D38" s="35"/>
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
@@ -30510,7 +30999,7 @@
       <c r="L38" s="36"/>
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B39" s="73"/>
+      <c r="B39" s="80"/>
       <c r="D39" s="35"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
@@ -30522,7 +31011,7 @@
       <c r="L39" s="36"/>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B40" s="73"/>
+      <c r="B40" s="80"/>
       <c r="D40" s="35"/>
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
@@ -30534,7 +31023,7 @@
       <c r="L40" s="36"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B41" s="73"/>
+      <c r="B41" s="80"/>
       <c r="D41" s="35"/>
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
@@ -30546,7 +31035,7 @@
       <c r="L41" s="36"/>
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B42" s="73"/>
+      <c r="B42" s="80"/>
       <c r="D42" s="35"/>
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
@@ -30558,7 +31047,7 @@
       <c r="L42" s="36"/>
     </row>
     <row r="43" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="74"/>
+      <c r="B43" s="81"/>
       <c r="D43" s="37"/>
       <c r="E43" s="38"/>
       <c r="F43" s="38"/>
@@ -30578,16 +31067,16 @@
       </c>
     </row>
     <row r="47" spans="2:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="D47" s="75" t="s">
+      <c r="D47" s="82" t="s">
         <v>424</v>
       </c>
-      <c r="E47" s="75"/>
-      <c r="F47" s="75"/>
-      <c r="G47" s="75"/>
-      <c r="H47" s="75"/>
+      <c r="E47" s="82"/>
+      <c r="F47" s="82"/>
+      <c r="G47" s="82"/>
+      <c r="H47" s="82"/>
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B48" s="72" t="s">
+      <c r="B48" s="79" t="s">
         <v>420</v>
       </c>
       <c r="D48" s="32" t="s">
@@ -30601,7 +31090,7 @@
       <c r="H48" s="40"/>
     </row>
     <row r="49" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B49" s="73"/>
+      <c r="B49" s="80"/>
       <c r="D49" s="35"/>
       <c r="E49" s="6"/>
       <c r="F49" s="6"/>
@@ -30609,7 +31098,7 @@
       <c r="H49" s="41"/>
     </row>
     <row r="50" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B50" s="73"/>
+      <c r="B50" s="80"/>
       <c r="D50" s="35"/>
       <c r="E50" s="6"/>
       <c r="F50" s="6"/>
@@ -30620,7 +31109,7 @@
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B51" s="73"/>
+      <c r="B51" s="80"/>
       <c r="D51" s="35"/>
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
@@ -30628,7 +31117,7 @@
       <c r="H51" s="41"/>
     </row>
     <row r="52" spans="2:11" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B52" s="74"/>
+      <c r="B52" s="81"/>
       <c r="D52" s="35"/>
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
@@ -30892,12 +31381,12 @@
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B93" s="71" t="s">
+      <c r="B93" s="78" t="s">
         <v>427</v>
       </c>
-      <c r="C93" s="71"/>
-      <c r="D93" s="71"/>
-      <c r="E93" s="71"/>
+      <c r="C93" s="78"/>
+      <c r="D93" s="78"/>
+      <c r="E93" s="78"/>
       <c r="F93" t="s">
         <v>428</v>
       </c>
@@ -31079,12 +31568,12 @@
       </c>
     </row>
     <row r="120" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B120" s="71" t="s">
+      <c r="B120" s="78" t="s">
         <v>432</v>
       </c>
-      <c r="C120" s="71"/>
-      <c r="D120" s="71"/>
-      <c r="E120" s="71"/>
+      <c r="C120" s="78"/>
+      <c r="D120" s="78"/>
+      <c r="E120" s="78"/>
     </row>
     <row r="122" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B122" t="s">
@@ -31360,20 +31849,20 @@
       </c>
     </row>
     <row r="150" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B150" s="71" t="s">
+      <c r="B150" s="78" t="s">
         <v>433</v>
       </c>
-      <c r="C150" s="71"/>
-      <c r="D150" s="71"/>
-      <c r="E150" s="71"/>
+      <c r="C150" s="78"/>
+      <c r="D150" s="78"/>
+      <c r="E150" s="78"/>
     </row>
     <row r="151" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B151" s="71" t="s">
+      <c r="B151" s="78" t="s">
         <v>434</v>
       </c>
-      <c r="C151" s="71"/>
-      <c r="D151" s="71"/>
-      <c r="E151" s="71"/>
+      <c r="C151" s="78"/>
+      <c r="D151" s="78"/>
+      <c r="E151" s="78"/>
     </row>
     <row r="153" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B153" t="s">
@@ -31488,12 +31977,12 @@
       </c>
     </row>
     <row r="168" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B168" s="71" t="s">
+      <c r="B168" s="78" t="s">
         <v>435</v>
       </c>
-      <c r="C168" s="71"/>
-      <c r="D168" s="71"/>
-      <c r="E168" s="71"/>
+      <c r="C168" s="78"/>
+      <c r="D168" s="78"/>
+      <c r="E168" s="78"/>
     </row>
     <row r="170" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B170" t="s">
@@ -31764,16 +32253,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B120:E120"/>
+    <mergeCell ref="B150:E150"/>
+    <mergeCell ref="B151:E151"/>
+    <mergeCell ref="B168:E168"/>
+    <mergeCell ref="H8:H11"/>
     <mergeCell ref="K8:K11"/>
     <mergeCell ref="B34:B43"/>
     <mergeCell ref="B48:B52"/>
     <mergeCell ref="D47:H47"/>
     <mergeCell ref="B93:E93"/>
-    <mergeCell ref="B120:E120"/>
-    <mergeCell ref="B150:E150"/>
-    <mergeCell ref="B151:E151"/>
-    <mergeCell ref="B168:E168"/>
-    <mergeCell ref="H8:H11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -32150,20 +32639,20 @@
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B44" s="71" t="s">
+      <c r="B44" s="78" t="s">
         <v>454</v>
       </c>
-      <c r="C44" s="71"/>
-      <c r="D44" s="71"/>
-      <c r="E44" s="71"/>
-      <c r="F44" s="71"/>
+      <c r="C44" s="78"/>
+      <c r="D44" s="78"/>
+      <c r="E44" s="78"/>
+      <c r="F44" s="78"/>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B45" s="71"/>
-      <c r="C45" s="71"/>
-      <c r="D45" s="71"/>
-      <c r="E45" s="71"/>
-      <c r="F45" s="71"/>
+      <c r="B45" s="78"/>
+      <c r="C45" s="78"/>
+      <c r="D45" s="78"/>
+      <c r="E45" s="78"/>
+      <c r="F45" s="78"/>
     </row>
     <row r="48" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B48" t="s">

</xml_diff>